<commit_message>
Add golden-path billing E2E + cross-role smoke suite + QA tooling
- Rebuild TC-E006/E008/E010 as the real two-step submit->approve->bill flow
  (golden path, unapproved-log guard, multi-log total) driven through the UI
- Add 16-test smoke suite: login per role, key page/form loads, role
  isolation, logout (@group smoke)
- Add Smoke sheet (TC-SM001..016) to qa/LD-Expert-QA.xlsx
- Fix flaky contract-form fill in QaAdminSessions (set end_date/no_show_rate
  explicitly instead of relying on racy auto-fill JS)
- Add qa() factory states (User/School) used by the QA suites
- Refresh QA commands/scripts/make targets + .gitattributes (*.sh eol=lf)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/qa/LD-Expert-QA.xlsx
+++ b/qa/LD-Expert-QA.xlsx
@@ -7,11 +7,12 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Admin" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Therapist" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Student" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finance" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E2E" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Smoke" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Admin" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Therapist" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Student" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finance" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E2E" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -23,7 +24,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="17">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -115,6 +116,9 @@
       <b val="1"/>
       <color rgb="FFFFFFFF"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="14">
@@ -231,7 +235,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -363,6 +367,7 @@
     <xf numFmtId="0" fontId="0" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1123,6 +1128,1087 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:P18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" style="44" min="1" max="1"/>
+    <col width="16" customWidth="1" style="44" min="2" max="2"/>
+    <col width="10" customWidth="1" style="44" min="3" max="3"/>
+    <col width="42" customWidth="1" style="44" min="4" max="4"/>
+    <col width="8" customWidth="1" style="44" min="5" max="5"/>
+    <col width="30" customWidth="1" style="44" min="6" max="6"/>
+    <col width="28" customWidth="1" style="44" min="7" max="7"/>
+    <col width="34" customWidth="1" style="44" min="8" max="8"/>
+    <col width="16" customWidth="1" style="44" min="9" max="9"/>
+    <col width="8" customWidth="1" style="44" min="10" max="10"/>
+    <col width="8" customWidth="1" style="44" min="11" max="11"/>
+    <col width="42" customWidth="1" style="44" min="12" max="12"/>
+    <col width="10" customWidth="1" style="44" min="13" max="13"/>
+    <col width="14" customWidth="1" style="44" min="14" max="14"/>
+    <col width="18" customWidth="1" style="44" min="15" max="15"/>
+    <col width="48" customWidth="1" style="44" min="16" max="16"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>LD Expert Bird - Smoke Test Cases (fast cross-role canary, @group smoke)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="49" t="inlineStr">
+        <is>
+          <t>TC ID</t>
+        </is>
+      </c>
+      <c r="B2" s="49" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="C2" s="49" t="inlineStr">
+        <is>
+          <t>Condition</t>
+        </is>
+      </c>
+      <c r="D2" s="49" t="inlineStr">
+        <is>
+          <t>Test Name</t>
+        </is>
+      </c>
+      <c r="E2" s="49" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="F2" s="49" t="inlineStr">
+        <is>
+          <t>Preconditions</t>
+        </is>
+      </c>
+      <c r="G2" s="49" t="inlineStr">
+        <is>
+          <t>Step 1</t>
+        </is>
+      </c>
+      <c r="H2" s="49" t="inlineStr">
+        <is>
+          <t>Step 2</t>
+        </is>
+      </c>
+      <c r="I2" s="49" t="inlineStr">
+        <is>
+          <t>Step 3</t>
+        </is>
+      </c>
+      <c r="J2" s="49" t="inlineStr">
+        <is>
+          <t>Step 4</t>
+        </is>
+      </c>
+      <c r="K2" s="49" t="inlineStr">
+        <is>
+          <t>Step 5</t>
+        </is>
+      </c>
+      <c r="L2" s="49" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="M2" s="49" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="N2" s="49" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="O2" s="49" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="P2" s="49" t="inlineStr">
+        <is>
+          <t>Dusk Test File</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>TC-SM001</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>App Health</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Valid</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Guest visiting home is redirected to login</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Logged out</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Navigate to /</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Observe redirect</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Redirected to /login; username and password fields visible</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>tests/BrowserQA/Smoke/QaAppSmokeBrowserTest.php</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>TC-SM002</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Authentication</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Valid</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Admin can log in via the login form</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Seeded system admin exists</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Navigate to /login</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Enter develop.ldexpert@gmail.com / Password123!</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Click Log in</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Redirected to /admin/dashboard</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>tests/BrowserQA/Smoke/QaAppSmokeBrowserTest.php</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>TC-SM003</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Authentication</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Valid</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Therapist can log in via the login form</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Therapist user + profile exist</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Navigate to /login</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Enter therapist username / password</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Click Log in</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Redirected to /therapist/dashboard</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>tests/BrowserQA/Smoke/QaAppSmokeBrowserTest.php</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>TC-SM004</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Authentication</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Valid</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Student can log in via the login form</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Student user exists</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Navigate to /login</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Enter student username / password</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Click Log in</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Redirected to /student/dashboard</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>tests/BrowserQA/Smoke/QaAppSmokeBrowserTest.php</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>TC-SM005</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Schools</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Valid</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Admin schools list loads</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Admin logged in</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Visit /admin/schools</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Page loads showing "Schools/Families", no error</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>tests/BrowserQA/Smoke/QaAppSmokeBrowserTest.php</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>TC-SM006</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Therapists</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Valid</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Admin therapists list loads</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Admin logged in</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Visit /admin/therapists</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Page loads showing "Therapists"</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>tests/BrowserQA/Smoke/QaAppSmokeBrowserTest.php</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>TC-SM007</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Students</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Valid</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Admin students list loads</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Admin logged in</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Visit /admin/students</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Page loads showing "Students"</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>tests/BrowserQA/Smoke/QaAppSmokeBrowserTest.php</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>TC-SM008</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Session Logs</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Valid</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Admin session logs list loads</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Admin logged in</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Visit /admin/session-logs</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Page loads showing "Session Logs"</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>tests/BrowserQA/Smoke/QaAppSmokeBrowserTest.php</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>TC-SM009</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Billing</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Valid</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Admin therapist bills list loads</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Admin logged in</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Visit /admin/billing/therapist-bills</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Page loads showing "Therapist Bills"</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>tests/BrowserQA/Smoke/QaAppSmokeBrowserTest.php</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>TC-SM010</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Valid</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Finance dashboard loads</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Admin logged in</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Visit /admin/finance/dashboard</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Page loads showing "Finance Dashboard"</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>tests/BrowserQA/Smoke/QaAppSmokeBrowserTest.php</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>TC-SM011</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Schools</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Valid</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>School create form opens</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Admin logged in</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Visit /admin/schools/create</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>Create form renders ("Add School/Family")</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>tests/BrowserQA/Smoke/QaAppSmokeBrowserTest.php</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>TC-SM012</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Students</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Valid</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Student create form opens</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Admin logged in</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Visit /admin/students/create</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>Create form renders ("Add Student")</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr"/>
+      <c r="O14" t="inlineStr"/>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>tests/BrowserQA/Smoke/QaAppSmokeBrowserTest.php</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>TC-SM013</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>SSA</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Valid</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Therapist SSAs page loads</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Therapist logged in</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Visit /therapist/ssas</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>Page loads showing "My SSAs"</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr"/>
+      <c r="O15" t="inlineStr"/>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>tests/BrowserQA/Smoke/QaAppSmokeBrowserTest.php</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>TC-SM014</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Access Control</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Invalid</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Student cannot access admin area</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Student logged in</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Visit /admin/dashboard</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>403 / redirected away (no admin content)</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr"/>
+      <c r="O16" t="inlineStr"/>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>tests/BrowserQA/Smoke/QaAppSmokeBrowserTest.php</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>TC-SM015</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Access Control</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Invalid</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Therapist cannot access admin area</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Therapist logged in</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Visit /admin/dashboard</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>403 / redirected away (no admin content)</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr"/>
+      <c r="O17" t="inlineStr"/>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>tests/BrowserQA/Smoke/QaAppSmokeBrowserTest.php</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>TC-SM016</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Authentication</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Valid</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Logged-in user can log out</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Admin logged in</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Submit the logout form</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Observe redirect</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>Redirected to /login</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr"/>
+      <c r="O18" t="inlineStr"/>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>tests/BrowserQA/Smoke/QaAppSmokeBrowserTest.php</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:T112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
@@ -7461,7 +8547,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -11065,7 +12151,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -11876,7 +12962,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -14938,7 +16024,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>